<commit_message>
Update on Macallan Image
</commit_message>
<xml_diff>
--- a/resources/5.10 最新价格.xlsx
+++ b/resources/5.10 最新价格.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Documents/Singapore/Plan &amp; Note Internship/Part Time/WeChatProjects/TrinityGlobe/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350DB398-5559-5143-8F4A-4B046FEB4DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667BAD5D-F3F2-CF44-A32D-D9B5670F6002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6820" yWindow="1000" windowWidth="28800" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -417,25 +417,25 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -704,10 +704,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="18" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -745,10 +745,10 @@
       <c r="Y1" s="2"/>
     </row>
     <row r="2" spans="1:25" ht="18" customHeight="1">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="11"/>
+      <c r="B2" s="9"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -774,10 +774,10 @@
       <c r="Y2" s="2"/>
     </row>
     <row r="3" spans="1:25" ht="18" customHeight="1">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="11"/>
+      <c r="B3" s="9"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2">
         <v>131</v>
@@ -811,10 +811,10 @@
       <c r="Y3" s="2"/>
     </row>
     <row r="4" spans="1:25" ht="18" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="11"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2">
         <v>147</v>
@@ -848,10 +848,10 @@
       <c r="Y4" s="2"/>
     </row>
     <row r="5" spans="1:25" ht="18" customHeight="1">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11"/>
+      <c r="B5" s="9"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2">
         <v>240</v>
@@ -885,10 +885,10 @@
       <c r="Y5" s="2"/>
     </row>
     <row r="6" spans="1:25" ht="18" customHeight="1">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="9"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2">
         <v>448</v>
@@ -922,10 +922,10 @@
       <c r="Y6" s="2"/>
     </row>
     <row r="7" spans="1:25" ht="18" customHeight="1">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="11"/>
+      <c r="B7" s="9"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2">
         <v>540</v>
@@ -959,10 +959,10 @@
       <c r="Y7" s="2"/>
     </row>
     <row r="8" spans="1:25" ht="18" customHeight="1">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="9"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2">
         <v>2800</v>
@@ -996,10 +996,10 @@
       <c r="Y8" s="2"/>
     </row>
     <row r="9" spans="1:25" ht="18" customHeight="1">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="11"/>
+      <c r="B9" s="9"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2">
         <v>4690</v>
@@ -1033,10 +1033,10 @@
       <c r="Y9" s="2"/>
     </row>
     <row r="10" spans="1:25" ht="18" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="11"/>
+      <c r="B10" s="9"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2">
         <v>6800</v>
@@ -1070,10 +1070,10 @@
       <c r="Y10" s="2"/>
     </row>
     <row r="11" spans="1:25" ht="18" customHeight="1">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="11"/>
+      <c r="B11" s="9"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -1099,10 +1099,10 @@
       <c r="Y11" s="2"/>
     </row>
     <row r="12" spans="1:25" ht="18" customHeight="1">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="11"/>
+      <c r="B12" s="9"/>
       <c r="C12" s="2">
         <v>129</v>
       </c>
@@ -1138,10 +1138,10 @@
       <c r="Y12" s="2"/>
     </row>
     <row r="13" spans="1:25" ht="18" customHeight="1">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="11"/>
+      <c r="B13" s="9"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2">
         <v>858</v>
@@ -1175,10 +1175,10 @@
       <c r="Y13" s="2"/>
     </row>
     <row r="14" spans="1:25" ht="18" customHeight="1">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="9"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2">
@@ -1210,10 +1210,10 @@
       <c r="Y14" s="2"/>
     </row>
     <row r="15" spans="1:25" ht="18" customHeight="1">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="11"/>
+      <c r="B15" s="9"/>
       <c r="C15" s="2">
         <v>237</v>
       </c>
@@ -1249,10 +1249,10 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:25" ht="18" customHeight="1">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="9"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2">
         <v>1038</v>
@@ -1286,10 +1286,10 @@
       <c r="Y16" s="2"/>
     </row>
     <row r="17" spans="1:25" ht="18" customHeight="1">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="11"/>
+      <c r="B17" s="9"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -1315,10 +1315,10 @@
       <c r="Y17" s="2"/>
     </row>
     <row r="18" spans="1:25" ht="18" customHeight="1">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="9"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2">
         <v>89</v>
@@ -1352,10 +1352,10 @@
       <c r="Y18" s="2"/>
     </row>
     <row r="19" spans="1:25" ht="18" customHeight="1">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="9"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2">
         <v>232</v>
@@ -1389,10 +1389,10 @@
       <c r="Y19" s="2"/>
     </row>
     <row r="20" spans="1:25" ht="18" customHeight="1">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="9"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2">
         <v>1398</v>
@@ -1426,10 +1426,10 @@
       <c r="Y20" s="2"/>
     </row>
     <row r="21" spans="1:25" ht="18" customHeight="1">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="9"/>
       <c r="C21" s="2">
         <v>77</v>
       </c>
@@ -1465,10 +1465,10 @@
       <c r="Y21" s="2"/>
     </row>
     <row r="22" spans="1:25" ht="18" customHeight="1">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="9"/>
       <c r="C22" s="2">
         <v>200</v>
       </c>
@@ -1504,10 +1504,10 @@
       <c r="Y22" s="2"/>
     </row>
     <row r="23" spans="1:25" ht="18" customHeight="1">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="9"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5">
@@ -1539,10 +1539,10 @@
       <c r="Y23" s="2"/>
     </row>
     <row r="24" spans="1:25" ht="18" customHeight="1">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="9"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5">
@@ -1574,10 +1574,10 @@
       <c r="Y24" s="2"/>
     </row>
     <row r="25" spans="1:25" ht="18" customHeight="1">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="9"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
@@ -1603,10 +1603,10 @@
       <c r="Y25" s="2"/>
     </row>
     <row r="26" spans="1:25" ht="18" customHeight="1">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="9"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2">
@@ -1639,10 +1639,10 @@
       <c r="Y26" s="2"/>
     </row>
     <row r="27" spans="1:25" ht="18" customHeight="1">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="11"/>
+      <c r="B27" s="9"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2">
@@ -1675,10 +1675,10 @@
       <c r="Y27" s="2"/>
     </row>
     <row r="28" spans="1:25" ht="18" customHeight="1">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="11"/>
+      <c r="B28" s="9"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2">
@@ -1711,10 +1711,10 @@
       <c r="Y28" s="2"/>
     </row>
     <row r="29" spans="1:25" ht="18" customHeight="1">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="11"/>
+      <c r="B29" s="9"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2">
@@ -1747,10 +1747,10 @@
       <c r="Y29" s="2"/>
     </row>
     <row r="30" spans="1:25" ht="18" customHeight="1">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="11"/>
+      <c r="B30" s="9"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2">
@@ -1783,10 +1783,10 @@
       <c r="Y30" s="2"/>
     </row>
     <row r="31" spans="1:25" ht="18" customHeight="1">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="11"/>
+      <c r="B31" s="9"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2">
@@ -1819,10 +1819,10 @@
       <c r="Y31" s="2"/>
     </row>
     <row r="32" spans="1:25" ht="18" customHeight="1">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="11"/>
+      <c r="B32" s="9"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2">
@@ -1855,10 +1855,10 @@
       <c r="Y32" s="2"/>
     </row>
     <row r="33" spans="1:25" ht="18" customHeight="1">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="11"/>
+      <c r="B33" s="9"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2">
@@ -1891,10 +1891,10 @@
       <c r="Y33" s="2"/>
     </row>
     <row r="34" spans="1:25" ht="18" customHeight="1">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="11"/>
+      <c r="B34" s="9"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2">
@@ -1927,10 +1927,10 @@
       <c r="Y34" s="2"/>
     </row>
     <row r="35" spans="1:25" ht="18" customHeight="1">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="11"/>
+      <c r="B35" s="9"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2">
@@ -1963,10 +1963,10 @@
       <c r="Y35" s="2"/>
     </row>
     <row r="36" spans="1:25" ht="18" customHeight="1">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="11"/>
+      <c r="B36" s="9"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2">
@@ -1999,10 +1999,10 @@
       <c r="Y36" s="2"/>
     </row>
     <row r="37" spans="1:25" ht="18" customHeight="1">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="11"/>
+      <c r="B37" s="9"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2">
@@ -2035,10 +2035,10 @@
       <c r="Y37" s="2"/>
     </row>
     <row r="38" spans="1:25" ht="18" customHeight="1">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="11"/>
+      <c r="B38" s="9"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2">
@@ -2071,10 +2071,10 @@
       <c r="Y38" s="2"/>
     </row>
     <row r="39" spans="1:25" ht="18" customHeight="1">
-      <c r="A39" s="13" t="s">
+      <c r="A39" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="11"/>
+      <c r="B39" s="9"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
@@ -2100,10 +2100,10 @@
       <c r="Y39" s="2"/>
     </row>
     <row r="40" spans="1:25" ht="18" customHeight="1">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="11"/>
+      <c r="B40" s="9"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2">
@@ -2136,10 +2136,10 @@
       <c r="Y40" s="2"/>
     </row>
     <row r="41" spans="1:25">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="11"/>
+      <c r="B41" s="9"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
@@ -2172,10 +2172,10 @@
       <c r="Y41" s="2"/>
     </row>
     <row r="42" spans="1:25">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="11"/>
+      <c r="B42" s="9"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2">
@@ -2208,10 +2208,10 @@
       <c r="Y42" s="2"/>
     </row>
     <row r="43" spans="1:25">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="11"/>
+      <c r="B43" s="9"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2">
@@ -2244,10 +2244,10 @@
       <c r="Y43" s="2"/>
     </row>
     <row r="44" spans="1:25">
-      <c r="A44" s="9" t="s">
+      <c r="A44" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="11"/>
+      <c r="B44" s="9"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2">
@@ -2280,10 +2280,10 @@
       <c r="Y44" s="2"/>
     </row>
     <row r="45" spans="1:25">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="11"/>
+      <c r="B45" s="9"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2">
@@ -2316,10 +2316,10 @@
       <c r="Y45" s="2"/>
     </row>
     <row r="46" spans="1:25">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="11"/>
+      <c r="B46" s="9"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2">
@@ -2352,10 +2352,10 @@
       <c r="Y46" s="2"/>
     </row>
     <row r="47" spans="1:25">
-      <c r="A47" s="9" t="s">
+      <c r="A47" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="11"/>
+      <c r="B47" s="9"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2">
@@ -2388,10 +2388,10 @@
       <c r="Y47" s="2"/>
     </row>
     <row r="48" spans="1:25">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="11"/>
+      <c r="B48" s="9"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2">
@@ -2424,10 +2424,10 @@
       <c r="Y48" s="2"/>
     </row>
     <row r="49" spans="1:25">
-      <c r="A49" s="9" t="s">
+      <c r="A49" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="11"/>
+      <c r="B49" s="9"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2">
@@ -2460,10 +2460,10 @@
       <c r="Y49" s="2"/>
     </row>
     <row r="50" spans="1:25">
-      <c r="A50" s="9" t="s">
+      <c r="A50" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B50" s="11"/>
+      <c r="B50" s="9"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2">
@@ -2496,10 +2496,10 @@
       <c r="Y50" s="2"/>
     </row>
     <row r="51" spans="1:25">
-      <c r="A51" s="9" t="s">
+      <c r="A51" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="11"/>
+      <c r="B51" s="9"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2">
@@ -2532,10 +2532,10 @@
       <c r="Y51" s="2"/>
     </row>
     <row r="52" spans="1:25">
-      <c r="A52" s="9" t="s">
+      <c r="A52" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="11"/>
+      <c r="B52" s="9"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2">
@@ -2568,10 +2568,10 @@
       <c r="Y52" s="2"/>
     </row>
     <row r="53" spans="1:25">
-      <c r="A53" s="9" t="s">
+      <c r="A53" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="11"/>
+      <c r="B53" s="9"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2">
@@ -2604,10 +2604,10 @@
       <c r="Y53" s="2"/>
     </row>
     <row r="54" spans="1:25">
-      <c r="A54" s="13" t="s">
+      <c r="A54" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B54" s="11"/>
+      <c r="B54" s="9"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
@@ -2633,10 +2633,10 @@
       <c r="Y54" s="2"/>
     </row>
     <row r="55" spans="1:25">
-      <c r="A55" s="9" t="s">
+      <c r="A55" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B55" s="11"/>
+      <c r="B55" s="9"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2">
@@ -2668,10 +2668,10 @@
       <c r="Y55" s="2"/>
     </row>
     <row r="56" spans="1:25">
-      <c r="A56" s="9" t="s">
+      <c r="A56" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B56" s="11"/>
+      <c r="B56" s="9"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2">
@@ -2703,10 +2703,10 @@
       <c r="Y56" s="2"/>
     </row>
     <row r="57" spans="1:25">
-      <c r="A57" s="9" t="s">
+      <c r="A57" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B57" s="11"/>
+      <c r="B57" s="9"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2">
@@ -2738,10 +2738,10 @@
       <c r="Y57" s="2"/>
     </row>
     <row r="58" spans="1:25">
-      <c r="A58" s="9" t="s">
+      <c r="A58" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B58" s="11"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2">
@@ -2773,10 +2773,10 @@
       <c r="Y58" s="2"/>
     </row>
     <row r="59" spans="1:25">
-      <c r="A59" s="9" t="s">
+      <c r="A59" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B59" s="11"/>
+      <c r="B59" s="9"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2">
         <v>228</v>
@@ -2810,10 +2810,10 @@
       <c r="Y59" s="2"/>
     </row>
     <row r="60" spans="1:25">
-      <c r="A60" s="9" t="s">
+      <c r="A60" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="11"/>
+      <c r="B60" s="9"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2">
         <v>340</v>
@@ -2847,10 +2847,10 @@
       <c r="Y60" s="2"/>
     </row>
     <row r="61" spans="1:25">
-      <c r="A61" s="9" t="s">
+      <c r="A61" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="11"/>
+      <c r="B61" s="9"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="4">
@@ -2882,10 +2882,10 @@
       <c r="Y61" s="2"/>
     </row>
     <row r="62" spans="1:25">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="11"/>
+      <c r="B62" s="9"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="4">
@@ -2917,10 +2917,10 @@
       <c r="Y62" s="2"/>
     </row>
     <row r="63" spans="1:25">
-      <c r="A63" s="9" t="s">
+      <c r="A63" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="11"/>
+      <c r="B63" s="9"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="4">
@@ -2952,10 +2952,10 @@
       <c r="Y63" s="2"/>
     </row>
     <row r="64" spans="1:25">
-      <c r="A64" s="9" t="s">
+      <c r="A64" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="11"/>
+      <c r="B64" s="9"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="4">
@@ -2987,10 +2987,10 @@
       <c r="Y64" s="2"/>
     </row>
     <row r="65" spans="1:25">
-      <c r="A65" s="13" t="s">
+      <c r="A65" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="11"/>
+      <c r="B65" s="9"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
@@ -3016,10 +3016,10 @@
       <c r="Y65" s="2"/>
     </row>
     <row r="66" spans="1:25">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="11"/>
+      <c r="B66" s="9"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2">
         <v>324</v>
@@ -3053,10 +3053,10 @@
       <c r="Y66" s="2"/>
     </row>
     <row r="67" spans="1:25">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="11"/>
+      <c r="B67" s="9"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2">
         <v>263</v>
@@ -3090,10 +3090,10 @@
       <c r="Y67" s="2"/>
     </row>
     <row r="68" spans="1:25">
-      <c r="A68" s="9" t="s">
+      <c r="A68" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B68" s="11"/>
+      <c r="B68" s="9"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2">
         <v>496</v>
@@ -3127,10 +3127,10 @@
       <c r="Y68" s="2"/>
     </row>
     <row r="69" spans="1:25">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B69" s="11"/>
+      <c r="B69" s="9"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2">
         <v>88</v>
@@ -3164,10 +3164,10 @@
       <c r="Y69" s="2"/>
     </row>
     <row r="70" spans="1:25">
-      <c r="A70" s="9" t="s">
+      <c r="A70" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="B70" s="11"/>
+      <c r="B70" s="9"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2">
         <v>116</v>
@@ -3201,10 +3201,10 @@
       <c r="Y70" s="2"/>
     </row>
     <row r="71" spans="1:25">
-      <c r="A71" s="9" t="s">
+      <c r="A71" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B71" s="11"/>
+      <c r="B71" s="9"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2">
         <v>124</v>
@@ -3238,10 +3238,10 @@
       <c r="Y71" s="2"/>
     </row>
     <row r="72" spans="1:25">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B72" s="11"/>
+      <c r="B72" s="9"/>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5">
@@ -3273,10 +3273,10 @@
       <c r="Y72" s="2"/>
     </row>
     <row r="73" spans="1:25">
-      <c r="A73" s="12" t="s">
+      <c r="A73" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B73" s="11"/>
+      <c r="B73" s="9"/>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5">
@@ -3308,10 +3308,10 @@
       <c r="Y73" s="2"/>
     </row>
     <row r="74" spans="1:25">
-      <c r="A74" s="12" t="s">
+      <c r="A74" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B74" s="11"/>
+      <c r="B74" s="9"/>
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
       <c r="E74" s="5">
@@ -3343,10 +3343,10 @@
       <c r="Y74" s="2"/>
     </row>
     <row r="75" spans="1:25">
-      <c r="A75" s="9" t="s">
+      <c r="A75" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B75" s="11"/>
+      <c r="B75" s="9"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2">
         <v>210</v>
@@ -3380,10 +3380,10 @@
       <c r="Y75" s="2"/>
     </row>
     <row r="76" spans="1:25">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B76" s="11"/>
+      <c r="B76" s="9"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="4">
@@ -3415,10 +3415,10 @@
       <c r="Y76" s="2"/>
     </row>
     <row r="77" spans="1:25">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B77" s="11"/>
+      <c r="B77" s="9"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="4">
@@ -3450,10 +3450,10 @@
       <c r="Y77" s="2"/>
     </row>
     <row r="78" spans="1:25">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B78" s="11"/>
+      <c r="B78" s="9"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="4">
@@ -3485,10 +3485,10 @@
       <c r="Y78" s="2"/>
     </row>
     <row r="79" spans="1:25">
-      <c r="A79" s="9" t="s">
+      <c r="A79" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B79" s="11"/>
+      <c r="B79" s="9"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="4">
@@ -3520,16 +3520,16 @@
       <c r="Y79" s="2"/>
     </row>
     <row r="80" spans="1:25">
-      <c r="A80" s="12" t="s">
+      <c r="A80" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="B80" s="11"/>
+      <c r="B80" s="9"/>
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5">
         <v>6</v>
       </c>
-      <c r="F80" s="10" t="s">
+      <c r="F80" s="14" t="s">
         <v>80</v>
       </c>
       <c r="G80" s="7">
@@ -3557,16 +3557,16 @@
       <c r="Y80" s="2"/>
     </row>
     <row r="81" spans="1:25">
-      <c r="A81" s="12" t="s">
+      <c r="A81" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B81" s="11"/>
+      <c r="B81" s="9"/>
       <c r="C81" s="5"/>
       <c r="D81" s="5"/>
       <c r="E81" s="5">
         <v>120</v>
       </c>
-      <c r="F81" s="10"/>
+      <c r="F81" s="14"/>
       <c r="G81" s="7">
         <v>6</v>
       </c>
@@ -7022,88 +7022,88 @@
     </row>
   </sheetData>
   <mergeCells count="82">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="F80:F81"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A81:B81"/>
     <mergeCell ref="A71:B71"/>
     <mergeCell ref="A62:B62"/>
     <mergeCell ref="A63:B63"/>
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="A65:B65"/>
     <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="F80:F81"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="A79:B79"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="A76:B76"/>
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="A68:B68"/>
     <mergeCell ref="A69:B69"/>
     <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>